<commit_message>
Tracker and detection confidence sweeps
</commit_message>
<xml_diff>
--- a/results/initial_benchmark_results.xlsx
+++ b/results/initial_benchmark_results.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10608"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10713"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jackmay/Desktop/KCF_YOLO/results/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{6B7DBA51-311D-7B46-9C1F-3047F6C30991}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EE376251-8D6A-0343-B68F-8657A820B398}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="20460" windowHeight="16380" activeTab="1" xr2:uid="{E79EF19B-9C5E-A944-86F5-B49891B7B6BC}"/>
+    <workbookView xWindow="3680" yWindow="1520" windowWidth="24740" windowHeight="14280" activeTab="1" xr2:uid="{E79EF19B-9C5E-A944-86F5-B49891B7B6BC}"/>
   </bookViews>
   <sheets>
     <sheet name="Standard" sheetId="2" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="35">
   <si>
     <t>Metrics</t>
   </si>
@@ -45,9 +45,6 @@
     <t>Nearest Neighbour</t>
   </si>
   <si>
-    <t>Hungarian Algo</t>
-  </si>
-  <si>
     <t>EMD Distance</t>
   </si>
   <si>
@@ -73,13 +70,85 @@
   </si>
   <si>
     <t>F1 Score</t>
+  </si>
+  <si>
+    <t>EMD HOG</t>
+  </si>
+  <si>
+    <t>deer_7</t>
+  </si>
+  <si>
+    <t>zebra_1</t>
+  </si>
+  <si>
+    <t>Hungarian Algo - Distance</t>
+  </si>
+  <si>
+    <t>Total Ground Truths: 4945</t>
+  </si>
+  <si>
+    <t>Hungarian Algo - HOG</t>
+  </si>
+  <si>
+    <t>True Positives: 4940</t>
+  </si>
+  <si>
+    <t>False Positives: 11</t>
+  </si>
+  <si>
+    <t>False Negatives: 0</t>
+  </si>
+  <si>
+    <t>Precision: 0.997778</t>
+  </si>
+  <si>
+    <t>Recall: 1</t>
+  </si>
+  <si>
+    <t>F1 Score: 0.998888</t>
+  </si>
+  <si>
+    <t>Hungarian Algo - IOU</t>
+  </si>
+  <si>
+    <t>Time (seconds)</t>
+  </si>
+  <si>
+    <t>Hungarian Algo - HOG / IOU</t>
+  </si>
+  <si>
+    <t>EMD Spatial Pool HOG</t>
+  </si>
+  <si>
+    <t>Total Ground Truths: 9901</t>
+  </si>
+  <si>
+    <t>True Positives: 8715</t>
+  </si>
+  <si>
+    <t>False Positives: 1185</t>
+  </si>
+  <si>
+    <t>False Negatives: 69</t>
+  </si>
+  <si>
+    <t>Precision: 0.880303</t>
+  </si>
+  <si>
+    <t>Recall: 0.992145</t>
+  </si>
+  <si>
+    <t>F1 Score: 0.932884</t>
+  </si>
+  <si>
+    <t>Elapsed time: 335.846 seconds</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -92,6 +161,13 @@
       <sz val="12"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FFFF0000"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
   </fonts>
@@ -210,8 +286,7 @@
   <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
@@ -219,6 +294,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -553,306 +629,627 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6E5C2320-C22A-5C40-A525-D5471DAB5458}">
-  <dimension ref="A1:E8"/>
+  <dimension ref="A1:H8"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="20.1640625" style="2" customWidth="1"/>
-    <col min="2" max="2" width="16.83203125" customWidth="1"/>
-    <col min="3" max="3" width="15.1640625" customWidth="1"/>
-    <col min="4" max="4" width="13.1640625" customWidth="1"/>
-    <col min="5" max="5" width="18.33203125" customWidth="1"/>
+    <col min="1" max="1" width="20.1640625" customWidth="1"/>
+    <col min="2" max="2" width="19.1640625" customWidth="1"/>
+    <col min="3" max="4" width="22.83203125" customWidth="1"/>
+    <col min="5" max="5" width="21.5" customWidth="1"/>
+    <col min="6" max="6" width="13.1640625" customWidth="1"/>
+    <col min="7" max="7" width="19.33203125" customWidth="1"/>
+    <col min="8" max="8" width="13.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" s="3" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="4" t="s">
+    <row r="1" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="5" t="s">
+      <c r="B1" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="5" t="s">
+      <c r="C1" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="E1" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="F1" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="5" t="s">
+      <c r="G1" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="6" t="s">
+      <c r="H1" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A2" s="6" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A2" s="7" t="s">
+      <c r="C2" t="s">
+        <v>15</v>
+      </c>
+      <c r="E2">
+        <v>4945</v>
+      </c>
+      <c r="H2" s="1">
+        <v>4945</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A3" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="B2" s="2">
-        <v>4945</v>
-      </c>
-      <c r="C2" s="2">
-        <v>4945</v>
-      </c>
-      <c r="D2" s="2">
-        <v>4945</v>
-      </c>
-      <c r="E2" s="1">
-        <v>4945</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A3" s="7" t="s">
+      <c r="C3" t="s">
+        <v>17</v>
+      </c>
+      <c r="E3">
+        <v>4940</v>
+      </c>
+      <c r="H3" s="1">
+        <v>4939</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A4" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="B3" s="2">
-        <v>4897</v>
-      </c>
-      <c r="C3" s="2">
-        <v>4897</v>
-      </c>
-      <c r="D3" s="2">
-        <v>4894</v>
-      </c>
-      <c r="E3" s="1">
-        <v>4897</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A4" s="7" t="s">
+      <c r="C4" t="s">
+        <v>18</v>
+      </c>
+      <c r="E4">
+        <v>11</v>
+      </c>
+      <c r="H4" s="1">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A5" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="B4" s="2">
-        <v>54</v>
-      </c>
-      <c r="C4" s="2">
-        <v>54</v>
-      </c>
-      <c r="D4" s="2">
-        <v>57</v>
-      </c>
-      <c r="E4" s="1">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A5" s="7" t="s">
+      <c r="C5" t="s">
+        <v>19</v>
+      </c>
+      <c r="E5">
+        <v>0</v>
+      </c>
+      <c r="H5" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A6" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="B5" s="2">
-        <v>43</v>
-      </c>
-      <c r="C5" s="2">
-        <v>43</v>
-      </c>
-      <c r="D5" s="2">
-        <v>45</v>
-      </c>
-      <c r="E5" s="1">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A6" s="7" t="s">
+      <c r="C6" t="s">
+        <v>20</v>
+      </c>
+      <c r="E6">
+        <v>0.99777800000000005</v>
+      </c>
+      <c r="H6" s="1">
+        <v>0.99757600000000002</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A7" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="B6" s="2">
-        <v>0.989093</v>
-      </c>
-      <c r="C6" s="2">
-        <v>0.989093</v>
-      </c>
-      <c r="D6" s="2">
-        <v>0.988487</v>
-      </c>
-      <c r="E6" s="1">
-        <v>0.989093</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A7" s="7" t="s">
+      <c r="C7" t="s">
+        <v>21</v>
+      </c>
+      <c r="E7">
+        <v>1</v>
+      </c>
+      <c r="H7" s="1">
+        <v>0.99979799999999996</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A8" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="B7" s="2">
-        <v>0.99129599999999995</v>
-      </c>
-      <c r="C7" s="2">
-        <v>0.99129599999999995</v>
-      </c>
-      <c r="D7" s="2">
-        <v>0.99088900000000002</v>
-      </c>
-      <c r="E7" s="1">
-        <v>0.99129599999999995</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A8" s="8" t="s">
-        <v>11</v>
-      </c>
-      <c r="B8" s="9">
-        <v>0.99019299999999999</v>
-      </c>
-      <c r="C8" s="9">
-        <v>0.99019299999999999</v>
-      </c>
-      <c r="D8" s="9">
-        <v>0.98968699999999998</v>
-      </c>
-      <c r="E8" s="10">
-        <v>0.99019299999999999</v>
+      <c r="B8" s="8"/>
+      <c r="C8" s="8" t="s">
+        <v>22</v>
+      </c>
+      <c r="D8" s="8"/>
+      <c r="E8" s="8">
+        <v>0.998888</v>
+      </c>
+      <c r="F8" s="8"/>
+      <c r="G8" s="8"/>
+      <c r="H8" s="9">
+        <v>0.99868599999999996</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AA8DF547-51E9-D048-9652-75EFE0641702}">
-  <dimension ref="A1:E8"/>
+  <dimension ref="A1:I30"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="20.1640625" style="2" customWidth="1"/>
-    <col min="2" max="2" width="16.83203125" customWidth="1"/>
-    <col min="3" max="3" width="15.1640625" customWidth="1"/>
-    <col min="4" max="4" width="13.1640625" customWidth="1"/>
-    <col min="5" max="5" width="18.33203125" customWidth="1"/>
+    <col min="1" max="1" width="20.1640625" customWidth="1"/>
+    <col min="2" max="2" width="21.33203125" customWidth="1"/>
+    <col min="3" max="3" width="22.33203125" customWidth="1"/>
+    <col min="4" max="4" width="22.5" customWidth="1"/>
+    <col min="5" max="5" width="21" customWidth="1"/>
+    <col min="6" max="6" width="22.83203125" customWidth="1"/>
+    <col min="7" max="7" width="18.33203125" customWidth="1"/>
+    <col min="8" max="8" width="19.1640625" customWidth="1"/>
+    <col min="9" max="9" width="20.1640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" s="3" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="4" t="s">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A1" s="10" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" s="2" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A2" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="5" t="s">
+      <c r="B2" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="5" t="s">
+      <c r="C2" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="D2" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="E2" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="F2" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="G2" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="5" t="s">
+      <c r="H2" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="6" t="s">
+      <c r="I2" s="5" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A3" s="6" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A2" s="7" t="s">
+      <c r="B3">
+        <v>4945</v>
+      </c>
+      <c r="C3">
+        <v>4945</v>
+      </c>
+      <c r="D3">
+        <v>4945</v>
+      </c>
+      <c r="E3">
+        <v>4945</v>
+      </c>
+      <c r="F3">
+        <v>4945</v>
+      </c>
+      <c r="I3" s="1">
+        <v>4945</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A4" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="B2" s="2">
-        <v>4945</v>
-      </c>
-      <c r="C2" s="2">
-        <v>4945</v>
-      </c>
-      <c r="D2" s="2">
-        <v>4945</v>
-      </c>
-      <c r="E2" s="1">
-        <v>4945</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A3" s="7" t="s">
+      <c r="B4">
+        <v>4834</v>
+      </c>
+      <c r="C4">
+        <v>4620</v>
+      </c>
+      <c r="D4">
+        <v>4657</v>
+      </c>
+      <c r="E4">
+        <v>4593</v>
+      </c>
+      <c r="F4">
+        <v>4657</v>
+      </c>
+      <c r="I4" s="1">
+        <v>4518</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A5" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="B3" s="2">
-        <v>4233</v>
-      </c>
-      <c r="C3" s="2">
-        <v>4246</v>
-      </c>
-      <c r="D3" s="2">
-        <v>4175</v>
-      </c>
-      <c r="E3" s="1">
-        <v>4252</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A4" s="7" t="s">
+      <c r="B5">
+        <v>117</v>
+      </c>
+      <c r="C5">
+        <v>331</v>
+      </c>
+      <c r="D5">
+        <v>294</v>
+      </c>
+      <c r="E5">
+        <v>358</v>
+      </c>
+      <c r="F5">
+        <v>294</v>
+      </c>
+      <c r="I5" s="1">
+        <v>433</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A6" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="B4" s="2">
-        <v>718</v>
-      </c>
-      <c r="C4" s="2">
-        <v>705</v>
-      </c>
-      <c r="D4" s="2">
-        <v>776</v>
-      </c>
-      <c r="E4" s="1">
-        <v>699</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A5" s="7" t="s">
+      <c r="B6">
+        <v>101</v>
+      </c>
+      <c r="C6">
+        <v>16</v>
+      </c>
+      <c r="D6">
+        <v>6</v>
+      </c>
+      <c r="E6">
+        <v>23</v>
+      </c>
+      <c r="F6">
+        <v>6</v>
+      </c>
+      <c r="I6" s="1">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A7" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="B5" s="2">
-        <v>61</v>
-      </c>
-      <c r="C5" s="2">
-        <v>53</v>
-      </c>
-      <c r="D5" s="2">
-        <v>86</v>
-      </c>
-      <c r="E5" s="1">
+      <c r="B7">
+        <v>0.97636800000000001</v>
+      </c>
+      <c r="C7">
+        <v>0.933145</v>
+      </c>
+      <c r="D7">
+        <v>0.94061799999999995</v>
+      </c>
+      <c r="E7">
+        <v>0.92769100000000004</v>
+      </c>
+      <c r="F7">
+        <v>0.94061799999999995</v>
+      </c>
+      <c r="I7" s="1">
+        <v>0.91254299999999999</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A8" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="B8">
+        <v>0.97953400000000002</v>
+      </c>
+      <c r="C8">
+        <v>0.99654900000000002</v>
+      </c>
+      <c r="D8">
+        <v>0.99871299999999996</v>
+      </c>
+      <c r="E8">
+        <v>0.99501700000000004</v>
+      </c>
+      <c r="F8">
+        <v>0.99871299999999996</v>
+      </c>
+      <c r="I8" s="1">
+        <v>0.99581200000000003</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A9" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="B9">
+        <v>0.97794899999999996</v>
+      </c>
+      <c r="C9">
+        <v>0.96380500000000002</v>
+      </c>
+      <c r="D9">
+        <v>0.96879499999999996</v>
+      </c>
+      <c r="E9">
+        <v>0.96017600000000003</v>
+      </c>
+      <c r="F9">
+        <v>0.96879499999999996</v>
+      </c>
+      <c r="I9" s="1">
+        <v>0.95236100000000001</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A10" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="B10" s="8">
+        <v>64.848600000000005</v>
+      </c>
+      <c r="C10" s="8">
+        <v>62.447899999999997</v>
+      </c>
+      <c r="D10" s="8">
+        <v>60.191499999999998</v>
+      </c>
+      <c r="E10" s="8">
+        <v>324.11599999999999</v>
+      </c>
+      <c r="F10" s="8">
+        <v>310.733</v>
+      </c>
+      <c r="G10" s="8"/>
+      <c r="H10" s="8"/>
+      <c r="I10" s="9">
+        <v>147.19499999999999</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A12" s="10" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A13" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="B13" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="C13" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="D13" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="E13" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="F13" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="G13" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="H13" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="I13" s="5" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A14" s="6" t="s">
+        <v>4</v>
+      </c>
+      <c r="D14">
+        <v>9901</v>
+      </c>
+      <c r="E14">
+        <v>9901</v>
+      </c>
+      <c r="F14">
+        <v>9901</v>
+      </c>
+      <c r="H14">
+        <v>9901</v>
+      </c>
+      <c r="I14" s="1">
+        <v>9901</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A15" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="D15">
+        <v>9508</v>
+      </c>
+      <c r="E15">
+        <v>9407</v>
+      </c>
+      <c r="F15">
+        <v>9508</v>
+      </c>
+      <c r="H15">
+        <v>9530</v>
+      </c>
+      <c r="I15" s="1">
+        <v>9380</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A16" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="D16">
+        <v>392</v>
+      </c>
+      <c r="E16">
+        <v>493</v>
+      </c>
+      <c r="F16">
+        <v>392</v>
+      </c>
+      <c r="H16">
+        <v>370</v>
+      </c>
+      <c r="I16" s="1">
+        <v>520</v>
+      </c>
+    </row>
+    <row r="17" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A17" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="D17">
         <v>37</v>
       </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A6" s="7" t="s">
+      <c r="E17">
+        <v>116</v>
+      </c>
+      <c r="F17">
+        <v>37</v>
+      </c>
+      <c r="H17">
+        <v>12</v>
+      </c>
+      <c r="I17" s="1">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="18" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A18" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="D18">
+        <v>0.96040400000000004</v>
+      </c>
+      <c r="E18">
+        <v>0.95020199999999999</v>
+      </c>
+      <c r="F18">
+        <v>0.96040400000000004</v>
+      </c>
+      <c r="H18">
+        <v>0.96262599999999998</v>
+      </c>
+      <c r="I18" s="1">
+        <v>0.94747499999999996</v>
+      </c>
+    </row>
+    <row r="19" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A19" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="B6" s="2">
-        <v>0.85497900000000004</v>
-      </c>
-      <c r="C6" s="2">
-        <v>0.85760499999999995</v>
-      </c>
-      <c r="D6" s="2">
-        <v>0.84326400000000001</v>
-      </c>
-      <c r="E6" s="1">
-        <v>0.85881600000000002</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A7" s="7" t="s">
+      <c r="D19">
+        <v>0.99612400000000001</v>
+      </c>
+      <c r="E19">
+        <v>0.987819</v>
+      </c>
+      <c r="F19">
+        <v>0.99612400000000001</v>
+      </c>
+      <c r="H19">
+        <v>0.99874200000000002</v>
+      </c>
+      <c r="I19" s="1">
+        <v>0.99417100000000003</v>
+      </c>
+    </row>
+    <row r="20" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A20" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="B7" s="2">
-        <v>0.98579399999999995</v>
-      </c>
-      <c r="C7" s="2">
-        <v>0.98767199999999999</v>
-      </c>
-      <c r="D7" s="2">
-        <v>0.97981700000000005</v>
-      </c>
-      <c r="E7" s="1">
-        <v>0.99137299999999995</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A8" s="8" t="s">
-        <v>11</v>
-      </c>
-      <c r="B8" s="9">
-        <v>0.91573800000000005</v>
-      </c>
-      <c r="C8" s="9">
-        <v>0.91805400000000004</v>
-      </c>
-      <c r="D8" s="9">
-        <v>0.90642599999999995</v>
-      </c>
-      <c r="E8" s="10">
-        <v>0.920346</v>
+      <c r="D20">
+        <v>0.97793799999999997</v>
+      </c>
+      <c r="E20">
+        <v>0.96864499999999998</v>
+      </c>
+      <c r="F20">
+        <v>0.97793799999999997</v>
+      </c>
+      <c r="H20">
+        <v>0.980352</v>
+      </c>
+      <c r="I20" s="1">
+        <v>0.97026100000000004</v>
+      </c>
+    </row>
+    <row r="21" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A21" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="B21" s="8"/>
+      <c r="C21" s="8"/>
+      <c r="D21" s="8">
+        <v>109.045</v>
+      </c>
+      <c r="E21" s="8">
+        <v>1360.5</v>
+      </c>
+      <c r="F21" s="8">
+        <v>983.17700000000002</v>
+      </c>
+      <c r="G21" s="8"/>
+      <c r="H21" s="8">
+        <v>136.07599999999999</v>
+      </c>
+      <c r="I21" s="9">
+        <v>146.38800000000001</v>
+      </c>
+    </row>
+    <row r="23" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="E23" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="24" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="E24" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="25" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="E25" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="26" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="E26" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="27" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="E27" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="28" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="E28" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="29" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="E29" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="30" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="E30" t="s">
+        <v>34</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
 </worksheet>
 </file>
</xml_diff>